<commit_message>
Finances: WhatsApp cost from Dec 2026, customers pay by bank transfer, ai-team.fr amount
</commit_message>
<xml_diff>
--- a/finances/IA-Factor-finances.xlsx
+++ b/finances/IA-Factor-finances.xlsx
@@ -814,7 +814,7 @@
     <row r="8">
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Coûts variables (IA par client…)</t>
+          <t>Coûts variables (IA, WhatsApp par client)</t>
         </is>
       </c>
       <c r="C8" s="8">
@@ -833,7 +833,7 @@
     <row r="9">
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Frais Stripe</t>
+          <t>Frais de paiement (virement : 0)</t>
         </is>
       </c>
       <c r="C9" s="8">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>Abonnement − coût variable − Stripe − cotisations</t>
+          <t>Abonnement − coût variable − frais de paiement − cotisations (hors WhatsApp)</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G29"/>
+  <dimension ref="B1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1504,30 +1504,30 @@
     <row r="24">
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Frais Stripe (% du paiement)</t>
+          <t>Frais de paiement (% du paiement)</t>
         </is>
       </c>
       <c r="C24" s="18" t="n">
-        <v>0.015</v>
+        <v>0</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Cartes UE, à vérifier</t>
+          <t>Clients payant par virement : 0. Si carte (Stripe) un jour : ~1,5 %</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Frais Stripe fixes par paiement (€)</t>
+          <t>Frais de paiement fixes par paiement (€)</t>
         </is>
       </c>
       <c r="C25" s="19" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="G25" s="11" t="inlineStr">
         <is>
-          <t>À vérifier</t>
+          <t>Virement : 0. Si carte (Stripe) : ~0,25 €</t>
         </is>
       </c>
     </row>
@@ -1588,6 +1588,36 @@
       <c r="G29" s="11" t="inlineStr">
         <is>
           <t>À vérifier : au-delà, facturer la TVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Coût WhatsApp par client Entreprise (€/mois)</t>
+        </is>
+      </c>
+      <c r="C30" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="11" t="inlineStr">
+        <is>
+          <t>Messages à l'initiative du commerce (rappels) ; réponses sous 24 h gratuites. Estimation 0,50–2 €, grille Meta à vérifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Début de WhatsApp (V2)</t>
+        </is>
+      </c>
+      <c r="C31" s="21" t="n">
+        <v>46357</v>
+      </c>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>Coût compté à partir de ce mois</t>
         </is>
       </c>
     </row>
@@ -1938,11 +1968,11 @@
         </is>
       </c>
       <c r="E8" s="23" t="n">
-        <v>0</v>
+        <v>10.25</v>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>€</t>
+          <t>$</t>
         </is>
       </c>
       <c r="G8" s="20">
@@ -1973,7 +2003,7 @@
       </c>
       <c r="N8" s="15" t="inlineStr">
         <is>
-          <t>À renseigner</t>
+          <t>Payé</t>
         </is>
       </c>
       <c r="O8" s="11" t="inlineStr">
@@ -3090,12 +3120,12 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Frais Stripe</t>
+          <t>Frais de paiement (virements des clients)</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Banque</t>
         </is>
       </c>
       <c r="D26" s="15" t="inlineStr">
@@ -3142,14 +3172,14 @@
       </c>
       <c r="O26" s="11" t="inlineStr">
         <is>
-          <t>Voir Paramètres : % + fixe par paiement</t>
+          <t>Les clients paient par virement : 0 € (voir Paramètres si carte un jour)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Paiement</t>
+          <t>IA</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -3189,10 +3219,12 @@
       </c>
       <c r="J27" s="15" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="K27" s="21" t="n"/>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="K27" s="21" t="n">
+        <v>46357</v>
+      </c>
       <c r="L27" s="21" t="n"/>
       <c r="M27" s="15" t="inlineStr">
         <is>
@@ -3206,7 +3238,7 @@
       </c>
       <c r="O27" s="11" t="inlineStr">
         <is>
-          <t>V2 seulement ; V1 sur Telegram : gratuit</t>
+          <t>Par client et par mois, à partir de décembre 2026 : voir Paramètres</t>
         </is>
       </c>
     </row>
@@ -4361,12 +4393,12 @@
       </c>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t>Coûts variables</t>
+          <t>Coûts variables (IA, WhatsApp)</t>
         </is>
       </c>
       <c r="N4" s="6" t="inlineStr">
         <is>
-          <t>Frais Stripe</t>
+          <t>Frais de paiement</t>
         </is>
       </c>
       <c r="O4" s="6" t="inlineStr">
@@ -4449,7 +4481,7 @@
         <v/>
       </c>
       <c r="M5" s="8">
-        <f>E5*'Paramètres'!$C$11+G5*'Paramètres'!$E$20+I5*'Paramètres'!$E$21</f>
+        <f>E5*'Paramètres'!$C$11+G5*'Paramètres'!$E$20+I5*'Paramètres'!$E$21+IF(B5&gt;='Paramètres'!$C$31,E5*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N5" s="8">
@@ -4529,7 +4561,7 @@
         <v/>
       </c>
       <c r="M6" s="8">
-        <f>E6*'Paramètres'!$C$11+G6*'Paramètres'!$E$20+I6*'Paramètres'!$E$21</f>
+        <f>E6*'Paramètres'!$C$11+G6*'Paramètres'!$E$20+I6*'Paramètres'!$E$21+IF(B6&gt;='Paramètres'!$C$31,E6*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N6" s="8">
@@ -4609,7 +4641,7 @@
         <v/>
       </c>
       <c r="M7" s="8">
-        <f>E7*'Paramètres'!$C$11+G7*'Paramètres'!$E$20+I7*'Paramètres'!$E$21</f>
+        <f>E7*'Paramètres'!$C$11+G7*'Paramètres'!$E$20+I7*'Paramètres'!$E$21+IF(B7&gt;='Paramètres'!$C$31,E7*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N7" s="8">
@@ -4689,7 +4721,7 @@
         <v/>
       </c>
       <c r="M8" s="8">
-        <f>E8*'Paramètres'!$C$11+G8*'Paramètres'!$E$20+I8*'Paramètres'!$E$21</f>
+        <f>E8*'Paramètres'!$C$11+G8*'Paramètres'!$E$20+I8*'Paramètres'!$E$21+IF(B8&gt;='Paramètres'!$C$31,E8*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N8" s="8">
@@ -4769,7 +4801,7 @@
         <v/>
       </c>
       <c r="M9" s="8">
-        <f>E9*'Paramètres'!$C$11+G9*'Paramètres'!$E$20+I9*'Paramètres'!$E$21</f>
+        <f>E9*'Paramètres'!$C$11+G9*'Paramètres'!$E$20+I9*'Paramètres'!$E$21+IF(B9&gt;='Paramètres'!$C$31,E9*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N9" s="8">
@@ -4849,7 +4881,7 @@
         <v/>
       </c>
       <c r="M10" s="8">
-        <f>E10*'Paramètres'!$C$11+G10*'Paramètres'!$E$20+I10*'Paramètres'!$E$21</f>
+        <f>E10*'Paramètres'!$C$11+G10*'Paramètres'!$E$20+I10*'Paramètres'!$E$21+IF(B10&gt;='Paramètres'!$C$31,E10*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N10" s="8">
@@ -4929,7 +4961,7 @@
         <v/>
       </c>
       <c r="M11" s="8">
-        <f>E11*'Paramètres'!$C$11+G11*'Paramètres'!$E$20+I11*'Paramètres'!$E$21</f>
+        <f>E11*'Paramètres'!$C$11+G11*'Paramètres'!$E$20+I11*'Paramètres'!$E$21+IF(B11&gt;='Paramètres'!$C$31,E11*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N11" s="8">
@@ -5009,7 +5041,7 @@
         <v/>
       </c>
       <c r="M12" s="8">
-        <f>E12*'Paramètres'!$C$11+G12*'Paramètres'!$E$20+I12*'Paramètres'!$E$21</f>
+        <f>E12*'Paramètres'!$C$11+G12*'Paramètres'!$E$20+I12*'Paramètres'!$E$21+IF(B12&gt;='Paramètres'!$C$31,E12*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N12" s="8">
@@ -5089,7 +5121,7 @@
         <v/>
       </c>
       <c r="M13" s="8">
-        <f>E13*'Paramètres'!$C$11+G13*'Paramètres'!$E$20+I13*'Paramètres'!$E$21</f>
+        <f>E13*'Paramètres'!$C$11+G13*'Paramètres'!$E$20+I13*'Paramètres'!$E$21+IF(B13&gt;='Paramètres'!$C$31,E13*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N13" s="8">
@@ -5169,7 +5201,7 @@
         <v/>
       </c>
       <c r="M14" s="8">
-        <f>E14*'Paramètres'!$C$11+G14*'Paramètres'!$E$20+I14*'Paramètres'!$E$21</f>
+        <f>E14*'Paramètres'!$C$11+G14*'Paramètres'!$E$20+I14*'Paramètres'!$E$21+IF(B14&gt;='Paramètres'!$C$31,E14*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N14" s="8">
@@ -5249,7 +5281,7 @@
         <v/>
       </c>
       <c r="M15" s="8">
-        <f>E15*'Paramètres'!$C$11+G15*'Paramètres'!$E$20+I15*'Paramètres'!$E$21</f>
+        <f>E15*'Paramètres'!$C$11+G15*'Paramètres'!$E$20+I15*'Paramètres'!$E$21+IF(B15&gt;='Paramètres'!$C$31,E15*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N15" s="8">
@@ -5329,7 +5361,7 @@
         <v/>
       </c>
       <c r="M16" s="8">
-        <f>E16*'Paramètres'!$C$11+G16*'Paramètres'!$E$20+I16*'Paramètres'!$E$21</f>
+        <f>E16*'Paramètres'!$C$11+G16*'Paramètres'!$E$20+I16*'Paramètres'!$E$21+IF(B16&gt;='Paramètres'!$C$31,E16*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N16" s="8">
@@ -5409,7 +5441,7 @@
         <v/>
       </c>
       <c r="M17" s="8">
-        <f>E17*'Paramètres'!$C$11+G17*'Paramètres'!$E$20+I17*'Paramètres'!$E$21</f>
+        <f>E17*'Paramètres'!$C$11+G17*'Paramètres'!$E$20+I17*'Paramètres'!$E$21+IF(B17&gt;='Paramètres'!$C$31,E17*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N17" s="8">
@@ -5489,7 +5521,7 @@
         <v/>
       </c>
       <c r="M18" s="8">
-        <f>E18*'Paramètres'!$C$11+G18*'Paramètres'!$E$20+I18*'Paramètres'!$E$21</f>
+        <f>E18*'Paramètres'!$C$11+G18*'Paramètres'!$E$20+I18*'Paramètres'!$E$21+IF(B18&gt;='Paramètres'!$C$31,E18*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N18" s="8">
@@ -5569,7 +5601,7 @@
         <v/>
       </c>
       <c r="M19" s="8">
-        <f>E19*'Paramètres'!$C$11+G19*'Paramètres'!$E$20+I19*'Paramètres'!$E$21</f>
+        <f>E19*'Paramètres'!$C$11+G19*'Paramètres'!$E$20+I19*'Paramètres'!$E$21+IF(B19&gt;='Paramètres'!$C$31,E19*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N19" s="8">
@@ -5649,7 +5681,7 @@
         <v/>
       </c>
       <c r="M20" s="8">
-        <f>E20*'Paramètres'!$C$11+G20*'Paramètres'!$E$20+I20*'Paramètres'!$E$21</f>
+        <f>E20*'Paramètres'!$C$11+G20*'Paramètres'!$E$20+I20*'Paramètres'!$E$21+IF(B20&gt;='Paramètres'!$C$31,E20*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N20" s="8">
@@ -5729,7 +5761,7 @@
         <v/>
       </c>
       <c r="M21" s="8">
-        <f>E21*'Paramètres'!$C$11+G21*'Paramètres'!$E$20+I21*'Paramètres'!$E$21</f>
+        <f>E21*'Paramètres'!$C$11+G21*'Paramètres'!$E$20+I21*'Paramètres'!$E$21+IF(B21&gt;='Paramètres'!$C$31,E21*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N21" s="8">
@@ -5809,7 +5841,7 @@
         <v/>
       </c>
       <c r="M22" s="8">
-        <f>E22*'Paramètres'!$C$11+G22*'Paramètres'!$E$20+I22*'Paramètres'!$E$21</f>
+        <f>E22*'Paramètres'!$C$11+G22*'Paramètres'!$E$20+I22*'Paramètres'!$E$21+IF(B22&gt;='Paramètres'!$C$31,E22*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N22" s="8">
@@ -5889,7 +5921,7 @@
         <v/>
       </c>
       <c r="M23" s="8">
-        <f>E23*'Paramètres'!$C$11+G23*'Paramètres'!$E$20+I23*'Paramètres'!$E$21</f>
+        <f>E23*'Paramètres'!$C$11+G23*'Paramètres'!$E$20+I23*'Paramètres'!$E$21+IF(B23&gt;='Paramètres'!$C$31,E23*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N23" s="8">
@@ -5969,7 +6001,7 @@
         <v/>
       </c>
       <c r="M24" s="8">
-        <f>E24*'Paramètres'!$C$11+G24*'Paramètres'!$E$20+I24*'Paramètres'!$E$21</f>
+        <f>E24*'Paramètres'!$C$11+G24*'Paramètres'!$E$20+I24*'Paramètres'!$E$21+IF(B24&gt;='Paramètres'!$C$31,E24*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N24" s="8">
@@ -6049,7 +6081,7 @@
         <v/>
       </c>
       <c r="M25" s="8">
-        <f>E25*'Paramètres'!$C$11+G25*'Paramètres'!$E$20+I25*'Paramètres'!$E$21</f>
+        <f>E25*'Paramètres'!$C$11+G25*'Paramètres'!$E$20+I25*'Paramètres'!$E$21+IF(B25&gt;='Paramètres'!$C$31,E25*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N25" s="8">
@@ -6129,7 +6161,7 @@
         <v/>
       </c>
       <c r="M26" s="8">
-        <f>E26*'Paramètres'!$C$11+G26*'Paramètres'!$E$20+I26*'Paramètres'!$E$21</f>
+        <f>E26*'Paramètres'!$C$11+G26*'Paramètres'!$E$20+I26*'Paramètres'!$E$21+IF(B26&gt;='Paramètres'!$C$31,E26*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N26" s="8">
@@ -6209,7 +6241,7 @@
         <v/>
       </c>
       <c r="M27" s="8">
-        <f>E27*'Paramètres'!$C$11+G27*'Paramètres'!$E$20+I27*'Paramètres'!$E$21</f>
+        <f>E27*'Paramètres'!$C$11+G27*'Paramètres'!$E$20+I27*'Paramètres'!$E$21+IF(B27&gt;='Paramètres'!$C$31,E27*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N27" s="8">
@@ -6289,7 +6321,7 @@
         <v/>
       </c>
       <c r="M28" s="8">
-        <f>E28*'Paramètres'!$C$11+G28*'Paramètres'!$E$20+I28*'Paramètres'!$E$21</f>
+        <f>E28*'Paramètres'!$C$11+G28*'Paramètres'!$E$20+I28*'Paramètres'!$E$21+IF(B28&gt;='Paramètres'!$C$31,E28*'Paramètres'!$C$30,0)</f>
         <v/>
       </c>
       <c r="N28" s="8">
@@ -6461,14 +6493,14 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>IA par client</t>
+          <t>IA et WhatsApp par client</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Charges : frais Stripe</t>
+          <t>Charges : frais de paiement</t>
         </is>
       </c>
       <c r="C7" s="8">
@@ -6849,10 +6881,12 @@
           <t>Domaine ai-team.fr</t>
         </is>
       </c>
-      <c r="C5" s="23" t="n"/>
+      <c r="C5" s="23" t="n">
+        <v>10.25</v>
+      </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>€</t>
+          <t>$</t>
         </is>
       </c>
       <c r="E5" s="20">
@@ -6871,7 +6905,7 @@
       </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
-          <t>Montant à renseigner</t>
+          <t>Non renouvelé</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">

</xml_diff>